<commit_message>
fix(phase7): Increase wait timeouts and element assertion resilience across test suites
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Summary_Report.xlsx
+++ b/automation/reports/Excel/Summary_Report.xlsx
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>470</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>63.83%</t>
         </is>
       </c>
     </row>

</xml_diff>